<commit_message>
Update MCH2008 homework grades
</commit_message>
<xml_diff>
--- a/MCH2008_homework.xlsx
+++ b/MCH2008_homework.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gökhan Gülser\Desktop\quiz_system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{028945DA-F23E-4D42-96AB-B4E15729205C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05580357-7FE2-4833-913D-DAAF64FB3008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2389,7 +2389,9 @@
       <c r="D2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="4"/>
+      <c r="E2" s="4">
+        <v>5</v>
+      </c>
       <c r="F2" s="4"/>
       <c r="G2" s="4" t="str">
         <f>IF('901'!F2="", "", '901'!F2)</f>
@@ -2417,7 +2419,9 @@
       <c r="D3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="4"/>
+      <c r="E3" s="4">
+        <v>47</v>
+      </c>
       <c r="F3" s="4"/>
       <c r="G3" s="4" t="str">
         <f>IF('901'!F3="", "", '901'!F3)</f>
@@ -2445,7 +2449,9 @@
       <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="4"/>
+      <c r="E4" s="4">
+        <v>1</v>
+      </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4" t="str">
         <f>IF('901'!F4="", "", '901'!F4)</f>
@@ -2473,7 +2479,9 @@
       <c r="D5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="4"/>
+      <c r="E5" s="4">
+        <v>4</v>
+      </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4" t="str">
         <f>IF('901'!F5="", "", '901'!F5)</f>
@@ -2501,7 +2509,9 @@
       <c r="D6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="4"/>
+      <c r="E6" s="4">
+        <v>2</v>
+      </c>
       <c r="F6" s="4"/>
       <c r="G6" s="4" t="str">
         <f>IF('901'!F6="", "", '901'!F6)</f>
@@ -2529,7 +2539,9 @@
       <c r="D7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="4"/>
+      <c r="E7" s="4">
+        <v>4</v>
+      </c>
       <c r="F7" s="4"/>
       <c r="G7" s="4" t="str">
         <f>IF('901'!F7="", "", '901'!F7)</f>
@@ -2557,7 +2569,9 @@
       <c r="D8" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="4"/>
+      <c r="E8" s="4">
+        <v>98</v>
+      </c>
       <c r="F8" s="4"/>
       <c r="G8" s="4" t="str">
         <f>IF('901'!F8="", "", '901'!F8)</f>
@@ -2585,7 +2599,9 @@
       <c r="D9" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="4"/>
+      <c r="E9" s="4">
+        <v>5</v>
+      </c>
       <c r="F9" s="4"/>
       <c r="G9" s="4" t="str">
         <f>IF('901'!F9="", "", '901'!F9)</f>
@@ -2613,7 +2629,9 @@
       <c r="D10" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E10" s="4"/>
+      <c r="E10" s="4">
+        <v>4</v>
+      </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="str">
         <f>IF('901'!F10="", "", '901'!F10)</f>
@@ -2641,7 +2659,9 @@
       <c r="D11" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E11" s="4"/>
+      <c r="E11" s="4">
+        <v>5</v>
+      </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="str">
         <f>IF('901'!F11="", "", '901'!F11)</f>
@@ -2669,7 +2689,9 @@
       <c r="D12" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E12" s="4"/>
+      <c r="E12" s="4">
+        <v>27</v>
+      </c>
       <c r="F12" s="4"/>
       <c r="G12" s="4" t="str">
         <f>IF('901'!F12="", "", '901'!F12)</f>
@@ -2697,7 +2719,9 @@
       <c r="D13" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="4"/>
+      <c r="E13" s="4">
+        <v>8</v>
+      </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="str">
         <f>IF('901'!F13="", "", '901'!F13)</f>

</xml_diff>

<commit_message>
Update portal app and homework records
</commit_message>
<xml_diff>
--- a/MCH2008_homework.xlsx
+++ b/MCH2008_homework.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gökhan Gülser\Desktop\quiz_system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{219FE4AF-613B-49A5-B719-5F2474112369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70922D30-968E-440E-AC09-4197C1DDDA61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1470" windowWidth="28800" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="901" sheetId="1" r:id="rId1"/>
@@ -2389,21 +2389,11 @@
       <c r="D2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="4">
-        <v>57</v>
-      </c>
-      <c r="F2" s="4">
-        <v>87</v>
-      </c>
-      <c r="G2" s="4">
-        <v>13</v>
-      </c>
-      <c r="H2" s="4">
-        <v>45</v>
-      </c>
-      <c r="I2" s="4">
-        <v>4</v>
-      </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
     </row>
     <row r="3" spans="1:9" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">

</xml_diff>